<commit_message>
Added two tests for correctness of movement of a dynamic object, and test whether a sprite or texture can be loaded.
</commit_message>
<xml_diff>
--- a/Test_Log.xlsx
+++ b/Test_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni Work\Angry Birds\angry-birds-clone-assignment-SubhamVala\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E64E7274-2526-45D5-BD0D-7971A086DCE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D804A962-19B6-42FD-9426-C4B476FD44FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
   </bookViews>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
   <si>
     <t>Date:</t>
   </si>
@@ -230,9 +230,6 @@
     <t>Fatal test for enemy health</t>
   </si>
   <si>
-    <t>if enemy is not dead.</t>
-  </si>
-  <si>
     <t>Non-Fatal test for max slingshot tension</t>
   </si>
   <si>
@@ -245,9 +242,6 @@
     <t>Non-Fatal test for bird type</t>
   </si>
   <si>
-    <t>birdtype should be red first.</t>
-  </si>
-  <si>
     <t>2b4a52516bf2059fc4d96345820601bdaf84a10f</t>
   </si>
   <si>
@@ -257,10 +251,31 @@
     <t>pigtype should be "pig", so normal pig</t>
   </si>
   <si>
-    <t>Fata test for if pig sprite textureRect is correct</t>
-  </si>
-  <si>
     <t>pig texture should only show the normal pig from the spritesheet</t>
+  </si>
+  <si>
+    <t>21/05/02026</t>
+  </si>
+  <si>
+    <t>6823a71668ee4a406b2891797d54d691468713bd</t>
+  </si>
+  <si>
+    <t>Fatal test for if pig sprite textureRect is correct</t>
+  </si>
+  <si>
+    <t>Fatal test to check if the position of the ground is correct in window.</t>
+  </si>
+  <si>
+    <t>ground position should be 400.0f and 590.0f.</t>
+  </si>
+  <si>
+    <t>Positions were originally in Box2D / Meters so had to convert back to SFML / Pixels before testing.</t>
+  </si>
+  <si>
+    <t>birdtype should be blue first.</t>
+  </si>
+  <si>
+    <t>if pig is not dead.</t>
   </si>
 </sst>
 </file>
@@ -909,7 +924,7 @@
         <v>8</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="G2" s="16" t="b">
         <v>1</v>
@@ -918,7 +933,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -933,13 +948,13 @@
         <v>11</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G3" s="9" t="b">
         <v>1</v>
@@ -948,7 +963,7 @@
         <v>1</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -963,13 +978,13 @@
         <v>11</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G4" s="9" t="b">
         <v>1</v>
@@ -978,7 +993,7 @@
         <v>1</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -990,16 +1005,16 @@
         <v>46162</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G5" s="9" t="b">
         <v>1</v>
@@ -1008,7 +1023,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1020,16 +1035,16 @@
         <v>46162</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G6" s="9" t="b">
         <v>1</v>
@@ -1038,7 +1053,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1046,14 +1061,30 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="12"/>
+      <c r="B7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1">

</xml_diff>

<commit_message>
Added three tests, testing if the pig is markedfordeletion before collided with bird, testing if bird has used abiltiy before user uses its ability, testing birdtype using the enum class.
</commit_message>
<xml_diff>
--- a/Test_Log.xlsx
+++ b/Test_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni Work\Angry Birds\angry-birds-clone-assignment-SubhamVala\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D804A962-19B6-42FD-9426-C4B476FD44FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F08EC5-612D-4F9B-9D83-66998118725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
+    <workbookView xWindow="5865" yWindow="2295" windowWidth="21600" windowHeight="11295" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Log" sheetId="1" r:id="rId1"/>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="42">
   <si>
     <t>Date:</t>
   </si>
@@ -239,9 +239,6 @@
     <t>None</t>
   </si>
   <si>
-    <t>Non-Fatal test for bird type</t>
-  </si>
-  <si>
     <t>2b4a52516bf2059fc4d96345820601bdaf84a10f</t>
   </si>
   <si>
@@ -276,6 +273,48 @@
   </si>
   <si>
     <t>if pig is not dead.</t>
+  </si>
+  <si>
+    <t>9761794bbae736dbc76b74d953f02fe23bb502df</t>
+  </si>
+  <si>
+    <t>Birds position xPos should increase and yPos should decrease. Means the bird moves towards the pigs.</t>
+  </si>
+  <si>
+    <t>Fatal and fixture test,  that takes the bird and launches it checking if it moves.</t>
+  </si>
+  <si>
+    <t>Fatal and Fixture test, checks to see if Sprites/Textures can be loaded.</t>
+  </si>
+  <si>
+    <t>if a sprite or texture of a sprite can be loaded, in this case it will be the blueBirds sprite.</t>
+  </si>
+  <si>
+    <t>world was not updated after launch. So added world.Step()</t>
+  </si>
+  <si>
+    <t>Non-Fatal test for bird type in slingshot</t>
+  </si>
+  <si>
+    <t>Non-Fatal test for birdtype using enum class</t>
+  </si>
+  <si>
+    <t>if the birdtype is blue using the enum class, which means it will have different values as a ball.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Non-Fatal test, on game start the bird should not have used ability.</t>
+  </si>
+  <si>
+    <t>If the bird has used its ability before the player has launched OR before the player enteres the ability key</t>
+  </si>
+  <si>
+    <t>Fatal test, on game start the pig should not be marked for deletion since it has not been collided with bird</t>
+  </si>
+  <si>
+    <t>if pig is marked for deletion on game start or before a bird collides</t>
   </si>
 </sst>
 </file>
@@ -924,7 +963,7 @@
         <v>8</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G2" s="16" t="b">
         <v>1</v>
@@ -978,13 +1017,13 @@
         <v>11</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G4" s="9" t="b">
         <v>1</v>
@@ -1005,16 +1044,16 @@
         <v>46162</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G5" s="9" t="b">
         <v>1</v>
@@ -1035,16 +1074,16 @@
         <v>46162</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G6" s="9" t="b">
         <v>1</v>
@@ -1062,19 +1101,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>22</v>
-      </c>
       <c r="D7" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G7" s="9" t="b">
         <v>1</v>
@@ -1083,7 +1122,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1091,70 +1130,144 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="12"/>
+      <c r="B8" s="3">
+        <v>46164</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="12"/>
+      <c r="B9" s="3">
+        <v>46164</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B10" s="3"/>
+      <c r="B10" s="3">
+        <v>46168</v>
+      </c>
       <c r="C10" s="9"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="12"/>
+      <c r="D10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B11" s="3"/>
+      <c r="B11" s="3">
+        <v>46168</v>
+      </c>
       <c r="C11" s="9"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="12"/>
+      <c r="D11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B12" s="3"/>
+      <c r="B12" s="3">
+        <v>46168</v>
+      </c>
       <c r="C12" s="9"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="12"/>
+      <c r="D12" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" s="12" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1195,7 +1308,9 @@
       <c r="E15" s="9"/>
       <c r="F15" s="6"/>
       <c r="G15" s="9"/>
-      <c r="H15" s="6"/>
+      <c r="H15" s="6" t="s">
+        <v>37</v>
+      </c>
       <c r="I15" s="12"/>
     </row>
     <row r="16" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added a test for position of the bluebird in relation to the plank, pig and catapul.
</commit_message>
<xml_diff>
--- a/Test_Log.xlsx
+++ b/Test_Log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni Work\Angry Birds\angry-birds-clone-assignment-SubhamVala\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Second_year\AngyBirds_Testing\angry-birds-clone-assignment-SubhamVala\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F08EC5-612D-4F9B-9D83-66998118725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{537DCE98-E47A-4C43-8FDD-5B863C824F86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5865" yWindow="2295" windowWidth="21600" windowHeight="11295" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Log" sheetId="1" r:id="rId1"/>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="45">
   <si>
     <t>Date:</t>
   </si>
@@ -315,6 +315,15 @@
   </si>
   <si>
     <t>if pig is marked for deletion on game start or before a bird collides</t>
+  </si>
+  <si>
+    <t>1f6237728d02778863d8d0750c8e706430e1037d</t>
+  </si>
+  <si>
+    <t>Non-Fatal test to check position of bluebird in relation of other objects</t>
+  </si>
+  <si>
+    <t>if birds xPos is less than the other Objects.</t>
   </si>
 </sst>
 </file>
@@ -1193,7 +1202,9 @@
       <c r="B10" s="3">
         <v>46168</v>
       </c>
-      <c r="C10" s="9"/>
+      <c r="C10" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="D10" s="6" t="s">
         <v>35</v>
       </c>
@@ -1221,7 +1232,9 @@
       <c r="B11" s="3">
         <v>46168</v>
       </c>
-      <c r="C11" s="9"/>
+      <c r="C11" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="D11" s="6" t="s">
         <v>38</v>
       </c>
@@ -1249,7 +1262,9 @@
       <c r="B12" s="3">
         <v>46168</v>
       </c>
-      <c r="C12" s="9"/>
+      <c r="C12" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="D12" s="6" t="s">
         <v>40</v>
       </c>
@@ -1274,14 +1289,28 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B13" s="3"/>
+      <c r="B13" s="3">
+        <v>46168</v>
+      </c>
       <c r="C13" s="9"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="12"/>
+      <c r="D13" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="1">

</xml_diff>

<commit_message>
Added a test for the correctness of the sequence of destuctors
</commit_message>
<xml_diff>
--- a/Test_Log.xlsx
+++ b/Test_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Second_year\AngyBirds_Testing\angry-birds-clone-assignment-SubhamVala\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{537DCE98-E47A-4C43-8FDD-5B863C824F86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7272CA2D-9C0D-4260-8E83-DA65721F788B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
+    <workbookView xWindow="6240" yWindow="900" windowWidth="21600" windowHeight="11295" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Log" sheetId="1" r:id="rId1"/>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="48">
   <si>
     <t>Date:</t>
   </si>
@@ -324,6 +324,15 @@
   </si>
   <si>
     <t>if birds xPos is less than the other Objects.</t>
+  </si>
+  <si>
+    <t>Fatal test on the correctness of the sequence of destructors</t>
+  </si>
+  <si>
+    <t>if the deconstructors are called in order from Pig -&gt; DynamicObject -&gt; GameObject</t>
+  </si>
+  <si>
+    <t>8418668bac44cfdd7a5109155d2d82e23527a00b</t>
   </si>
 </sst>
 </file>
@@ -1292,7 +1301,9 @@
       <c r="B13" s="3">
         <v>46168</v>
       </c>
-      <c r="C13" s="9"/>
+      <c r="C13" s="9" t="s">
+        <v>47</v>
+      </c>
       <c r="D13" s="6" t="s">
         <v>43</v>
       </c>
@@ -1317,14 +1328,28 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B14" s="3"/>
+      <c r="B14" s="3">
+        <v>46169</v>
+      </c>
       <c r="C14" s="9"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="12"/>
+      <c r="D14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" s="12" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="1">

</xml_diff>

<commit_message>
Final commit for Tests.
</commit_message>
<xml_diff>
--- a/Test_Log.xlsx
+++ b/Test_Log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Second_year\AngyBirds_Testing\angry-birds-clone-assignment-SubhamVala\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni Work\Angry Birds\angry-birds-clone-assignment-SubhamVala\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6BCBC3-B71E-42AB-B248-1DAD00E84EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58DC8353-7697-40CD-B03B-ACC769C50449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6240" yWindow="900" windowWidth="21600" windowHeight="11295" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Log" sheetId="1" r:id="rId1"/>
@@ -230,9 +230,6 @@
     <t>Fatal test for enemy health</t>
   </si>
   <si>
-    <t>Non-Fatal test for max slingshot tension</t>
-  </si>
-  <si>
     <t>if slingshot is less than max tension</t>
   </si>
   <si>
@@ -263,9 +260,6 @@
     <t>Fatal test to check if the position of the ground is correct in window.</t>
   </si>
   <si>
-    <t>ground position should be 400.0f and 590.0f.</t>
-  </si>
-  <si>
     <t>Positions were originally in Box2D / Meters so had to convert back to SFML / Pixels before testing.</t>
   </si>
   <si>
@@ -293,9 +287,6 @@
     <t>world was not updated after launch. So added world.Step()</t>
   </si>
   <si>
-    <t>Non-Fatal test for bird type in slingshot</t>
-  </si>
-  <si>
     <t>Non-Fatal test for birdtype using enum class</t>
   </si>
   <si>
@@ -336,6 +327,15 @@
   </si>
   <si>
     <t>473ba50ff7ca4a26e5787a779c69ac613e62be8a</t>
+  </si>
+  <si>
+    <t>Non-Fatal test for max slingshot tension function in slingshot.h</t>
+  </si>
+  <si>
+    <t>Non-Fatal test for bird type in slingshot.h</t>
+  </si>
+  <si>
+    <t>ground position should be 400.0f and 590.0f, so it should be less than 800.0f, 600.0f,</t>
   </si>
 </sst>
 </file>
@@ -984,7 +984,7 @@
         <v>8</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G2" s="16" t="b">
         <v>1</v>
@@ -993,7 +993,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1008,22 +1008,22 @@
         <v>11</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="12" t="s">
         <v>14</v>
-      </c>
-      <c r="G3" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1038,13 +1038,13 @@
         <v>11</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G4" s="9" t="b">
         <v>1</v>
@@ -1053,7 +1053,7 @@
         <v>1</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1065,16 +1065,16 @@
         <v>46162</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>16</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>17</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G5" s="9" t="b">
         <v>1</v>
@@ -1083,7 +1083,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1095,16 +1095,16 @@
         <v>46162</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G6" s="9" t="b">
         <v>1</v>
@@ -1113,7 +1113,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1122,19 +1122,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>21</v>
-      </c>
       <c r="D7" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="G7" s="9" t="b">
         <v>1</v>
@@ -1143,7 +1143,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1155,16 +1155,16 @@
         <v>46164</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>7</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G8" s="9" t="b">
         <v>1</v>
@@ -1173,7 +1173,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1185,16 +1185,16 @@
         <v>46164</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G9" s="9" t="b">
         <v>1</v>
@@ -1203,7 +1203,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1215,16 +1215,16 @@
         <v>46168</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G10" s="9" t="b">
         <v>1</v>
@@ -1233,7 +1233,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1245,16 +1245,16 @@
         <v>46168</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G11" s="9" t="b">
         <v>0</v>
@@ -1263,7 +1263,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1275,16 +1275,16 @@
         <v>46168</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G12" s="9" t="b">
         <v>0</v>
@@ -1293,7 +1293,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1305,16 +1305,16 @@
         <v>46168</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="G13" s="9" t="b">
         <v>1</v>
@@ -1323,7 +1323,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1335,16 +1335,16 @@
         <v>46169</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>7</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G14" s="9" t="b">
         <v>1</v>
@@ -1353,7 +1353,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1368,7 +1368,7 @@
       <c r="F15" s="6"/>
       <c r="G15" s="9"/>
       <c r="H15" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="I15" s="12"/>
     </row>

</xml_diff>